<commit_message>
Update roster points: batt2 الطيرة 122 + الدور 35; Attendance.html fallback in sync
</commit_message>
<xml_diff>
--- a/roster.xlsx
+++ b/roster.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BASEL\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BASEL\Desktop\نظام تفقد\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EFDB97B-6827-434A-9964-204F4AB162E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217EE8C9-1373-498F-9EB2-8ADDC2F07667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E3E8A68-987D-4C06-BFB9-2CF7CF2E1A8C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="885">
   <si>
     <t>الجهة الفرعية</t>
   </si>
@@ -2691,6 +2691,9 @@
   </si>
   <si>
     <t>الطيرة</t>
+  </si>
+  <si>
+    <t>الدور</t>
   </si>
 </sst>
 </file>
@@ -2862,15 +2865,7 @@
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="37">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -9830,7 +9825,7 @@
         <v>601</v>
       </c>
       <c r="F261" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G261" s="16" t="s">
         <v>657</v>
@@ -9854,7 +9849,7 @@
         <v>601</v>
       </c>
       <c r="F262" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G262" s="16" t="s">
         <v>647</v>
@@ -9878,7 +9873,7 @@
         <v>601</v>
       </c>
       <c r="F263" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G263" s="16" t="s">
         <v>611</v>
@@ -9902,7 +9897,7 @@
         <v>601</v>
       </c>
       <c r="F264" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G264" s="16" t="s">
         <v>732</v>
@@ -9926,7 +9921,7 @@
         <v>601</v>
       </c>
       <c r="F265" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G265" s="16" t="s">
         <v>621</v>
@@ -9950,7 +9945,7 @@
         <v>601</v>
       </c>
       <c r="F266" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G266" s="16" t="s">
         <v>856</v>
@@ -9974,7 +9969,7 @@
         <v>601</v>
       </c>
       <c r="F267" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G267" s="16" t="s">
         <v>749</v>
@@ -9998,7 +9993,7 @@
         <v>601</v>
       </c>
       <c r="F268" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G268" s="16" t="s">
         <v>792</v>
@@ -10022,7 +10017,7 @@
         <v>601</v>
       </c>
       <c r="F269" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G269" s="16" t="s">
         <v>784</v>
@@ -10046,7 +10041,7 @@
         <v>601</v>
       </c>
       <c r="F270" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G270" s="16" t="s">
         <v>842</v>
@@ -10070,7 +10065,7 @@
         <v>601</v>
       </c>
       <c r="F271" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G271" s="12"/>
       <c r="J271" s="6"/>
@@ -10092,7 +10087,7 @@
         <v>601</v>
       </c>
       <c r="F272" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G272" s="16" t="s">
         <v>660</v>
@@ -10116,7 +10111,7 @@
         <v>601</v>
       </c>
       <c r="F273" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G273" s="16" t="s">
         <v>733</v>
@@ -10140,7 +10135,7 @@
         <v>601</v>
       </c>
       <c r="F274" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G274" s="16" t="s">
         <v>747</v>
@@ -10164,7 +10159,7 @@
         <v>601</v>
       </c>
       <c r="F275" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G275" s="16" t="s">
         <v>880</v>
@@ -10188,7 +10183,7 @@
         <v>601</v>
       </c>
       <c r="F276" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G276" s="16" t="s">
         <v>725</v>
@@ -10212,7 +10207,7 @@
         <v>601</v>
       </c>
       <c r="F277" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G277" s="16" t="s">
         <v>765</v>
@@ -10236,7 +10231,7 @@
         <v>601</v>
       </c>
       <c r="F278" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G278" s="16" t="s">
         <v>730</v>
@@ -10260,7 +10255,7 @@
         <v>601</v>
       </c>
       <c r="F279" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G279" s="16" t="s">
         <v>877</v>
@@ -10284,7 +10279,7 @@
         <v>601</v>
       </c>
       <c r="F280" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G280" s="16" t="s">
         <v>752</v>
@@ -10308,7 +10303,7 @@
         <v>601</v>
       </c>
       <c r="F281" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G281" s="16" t="s">
         <v>672</v>
@@ -10332,7 +10327,7 @@
         <v>601</v>
       </c>
       <c r="F282" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G282" s="16" t="s">
         <v>793</v>
@@ -10356,7 +10351,7 @@
         <v>601</v>
       </c>
       <c r="F283" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G283" s="16" t="s">
         <v>683</v>
@@ -10380,7 +10375,7 @@
         <v>601</v>
       </c>
       <c r="F284" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G284" s="16" t="s">
         <v>743</v>
@@ -10404,7 +10399,7 @@
         <v>601</v>
       </c>
       <c r="F285" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G285" s="16" t="s">
         <v>850</v>
@@ -10428,7 +10423,7 @@
         <v>601</v>
       </c>
       <c r="F286" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G286" s="16" t="s">
         <v>642</v>
@@ -10452,7 +10447,7 @@
         <v>601</v>
       </c>
       <c r="F287" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G287" s="16" t="s">
         <v>717</v>
@@ -10476,7 +10471,7 @@
         <v>601</v>
       </c>
       <c r="F288" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G288" s="16" t="s">
         <v>871</v>
@@ -10500,7 +10495,7 @@
         <v>601</v>
       </c>
       <c r="F289" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G289" s="16" t="s">
         <v>855</v>
@@ -10524,7 +10519,7 @@
         <v>601</v>
       </c>
       <c r="F290" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G290" s="16" t="s">
         <v>840</v>
@@ -10548,7 +10543,7 @@
         <v>601</v>
       </c>
       <c r="F291" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G291" s="16" t="s">
         <v>680</v>
@@ -10572,7 +10567,7 @@
         <v>601</v>
       </c>
       <c r="F292" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G292" s="16" t="s">
         <v>678</v>
@@ -10596,7 +10591,7 @@
         <v>601</v>
       </c>
       <c r="F293" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G293" s="16" t="s">
         <v>741</v>
@@ -10620,7 +10615,7 @@
         <v>601</v>
       </c>
       <c r="F294" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G294" s="16" t="s">
         <v>758</v>
@@ -10644,7 +10639,7 @@
         <v>601</v>
       </c>
       <c r="F295" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G295" s="16" t="s">
         <v>725</v>
@@ -10654,63 +10649,63 @@
   </sheetData>
   <autoFilter ref="A1:G295" xr:uid="{9F38B8BA-4557-470F-96FC-6D7AF2400F22}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G138">
-      <sortCondition sortBy="cellColor" ref="D1:D295" dxfId="37"/>
+      <sortCondition sortBy="cellColor" ref="D1:D295" dxfId="36"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="36" priority="275"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="275"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A295">
+    <cfRule type="duplicateValues" dxfId="34" priority="560"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="561"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="562"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="563"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="564"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="565"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="566"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A295">
+    <cfRule type="duplicateValues" dxfId="27" priority="574"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="575"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="576"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="577"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="35" priority="320"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="320"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C295">
+    <cfRule type="duplicateValues" dxfId="22" priority="584"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="586"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="585"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="582"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="583"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="587"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="588"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="589"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="590"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="591"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="592"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="593"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="594"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="595"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="596"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="597"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C295">
+    <cfRule type="duplicateValues" dxfId="6" priority="617"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="614"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="615"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="616"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C284:C295">
-    <cfRule type="duplicateValues" dxfId="34" priority="536"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="536"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:D1048576">
-    <cfRule type="duplicateValues" dxfId="33" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:G1">
-    <cfRule type="duplicateValues" dxfId="32" priority="321"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A295">
-    <cfRule type="duplicateValues" dxfId="31" priority="560"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="561"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="562"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="563"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="564"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="565"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="566"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A295">
-    <cfRule type="duplicateValues" dxfId="24" priority="574"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="575"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="576"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="577"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C295">
-    <cfRule type="duplicateValues" dxfId="20" priority="582"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="583"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="584"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="585"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="586"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="587"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="588"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="589"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="590"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="591"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="592"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="593"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="594"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="595"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="596"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="597"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C295">
-    <cfRule type="duplicateValues" dxfId="4" priority="614"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="615"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="616"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="617"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="321"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>